<commit_message>
Update bug report file with new changes
</commit_message>
<xml_diff>
--- a/QA_report/bug_report.xlsx
+++ b/QA_report/bug_report.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="28">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="31">
   <si>
     <t>BUG ID</t>
   </si>
@@ -114,6 +114,15 @@
   </si>
   <si>
     <t>Suggestion: The Not started projects should be grayed out</t>
+  </si>
+  <si>
+    <t>3a</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Data is not persisting </t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Change the state of a Task and refeash </t>
   </si>
 </sst>
 </file>
@@ -434,7 +443,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A2:H8"/>
+  <dimension ref="A2:H9"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="27.6640625" style="1" customWidth="1"/>
@@ -489,6 +498,9 @@
       <c r="F3" s="1" t="s">
         <v>16</v>
       </c>
+      <c r="H3" s="1" t="s">
+        <v>28</v>
+      </c>
     </row>
     <row r="4" spans="1:8" ht="72" x14ac:dyDescent="0.3">
       <c r="A4">
@@ -597,6 +609,26 @@
       </c>
       <c r="F8" s="1" t="s">
         <v>26</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" ht="43.2" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A9">
+        <v>7</v>
+      </c>
+      <c r="B9" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="C9" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D9" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="E9" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="F9" s="1" t="s">
+        <v>16</v>
       </c>
     </row>
   </sheetData>

</xml_diff>